<commit_message>
fix kết xuất thuế
</commit_message>
<xml_diff>
--- a/BackEnd/Server/Controllers/FastReport/TaxTemplates/Mau_Phieu_chi_tvt.xlsx
+++ b/BackEnd/Server/Controllers/FastReport/TaxTemplates/Mau_Phieu_chi_tvt.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\BUSINESS DEVELOPMENT\PHAM MEM SAO BAC DAU\UP PM THUE\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{764FA01A-8E94-4786-AC72-12F6666DC7ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-60" yWindow="-60" windowWidth="19320" windowHeight="14880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-60" yWindow="-60" windowWidth="19320" windowHeight="12220"/>
   </bookViews>
   <sheets>
     <sheet name="CT" sheetId="1" r:id="rId1"/>
@@ -34,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Ma_vv</t>
   </si>
@@ -81,9 +75,6 @@
     <t>Ma_dvcs</t>
   </si>
   <si>
-    <t>CONGTY</t>
-  </si>
-  <si>
     <t>Ngµy CT</t>
   </si>
   <si>
@@ -106,66 +97,12 @@
   </si>
   <si>
     <t>Ngµy H§</t>
-  </si>
-  <si>
-    <t>13311</t>
-  </si>
-  <si>
-    <t>0301452948</t>
-  </si>
-  <si>
-    <t>11211</t>
-  </si>
-  <si>
-    <t>11210</t>
-  </si>
-  <si>
-    <t>0100111948-099</t>
-  </si>
-  <si>
-    <t>Lai cong don: 6,482,192 VND</t>
-  </si>
-  <si>
-    <t>6352</t>
-  </si>
-  <si>
-    <t>K26TBB</t>
-  </si>
-  <si>
-    <t>4047</t>
-  </si>
-  <si>
-    <t>ng©n hµng th­¬ng m¹i cæ phÇn c«ng th­¬ng viÖt nam - chi nh¸nh bÕn løc</t>
-  </si>
-  <si>
-    <t>Sè 159 Quèc lé 1A Khu phè 1, ThÞ TrÊn BÕn Løc, HuyÖn BÕn Løc, TØnh Long An, ViÖt Nam</t>
-  </si>
-  <si>
-    <t>TRICH THU TIEN VAY - LAI</t>
-  </si>
-  <si>
-    <t>K26TYY</t>
-  </si>
-  <si>
-    <t>296844</t>
-  </si>
-  <si>
-    <t>ng©n hµng th­¬ng m¹i cæ phÇn ¸ ch©u</t>
-  </si>
-  <si>
-    <t>442 NguyÔn ThÞ Minh Khai, Ph­êng 5, QuËn 3, TP Hå ChÝ Minh</t>
-  </si>
-  <si>
-    <t>CIC0126042</t>
-  </si>
-  <si>
-    <t>CIC0126043</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
@@ -298,7 +235,7 @@
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 5" xfId="2" xr:uid="{401DCD63-B776-446F-9737-0DB650AE3563}"/>
+    <cellStyle name="Normal 5" xfId="2"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -314,9 +251,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -354,7 +291,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -426,7 +363,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -599,53 +536,53 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:W106"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" style="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" style="13" customWidth="1"/>
-    <col min="4" max="4" width="19.42578125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="16.85546875" style="13" customWidth="1"/>
-    <col min="6" max="6" width="29.5703125" style="13" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" style="7" customWidth="1"/>
-    <col min="8" max="8" width="12.28515625" style="7" customWidth="1"/>
+    <col min="1" max="1" width="14.453125" style="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7265625" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.81640625" style="13" customWidth="1"/>
+    <col min="4" max="4" width="19.453125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="16.81640625" style="13" customWidth="1"/>
+    <col min="6" max="6" width="29.54296875" style="13" customWidth="1"/>
+    <col min="7" max="7" width="14.54296875" style="7" customWidth="1"/>
+    <col min="8" max="8" width="12.26953125" style="7" customWidth="1"/>
     <col min="9" max="9" width="14" style="15" customWidth="1"/>
-    <col min="10" max="11" width="8.85546875" style="4"/>
-    <col min="12" max="12" width="12.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.140625" style="13" customWidth="1"/>
-    <col min="15" max="15" width="8.85546875" style="13"/>
-    <col min="16" max="16" width="11.28515625" style="10" customWidth="1"/>
+    <col min="10" max="11" width="8.81640625" style="4"/>
+    <col min="12" max="12" width="12.7265625" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.1796875" style="13" customWidth="1"/>
+    <col min="15" max="15" width="8.81640625" style="13"/>
+    <col min="16" max="16" width="11.26953125" style="10" customWidth="1"/>
     <col min="17" max="17" width="17" style="13" customWidth="1"/>
-    <col min="18" max="18" width="8.85546875" style="13"/>
-    <col min="19" max="19" width="46.28515625" style="13" customWidth="1"/>
-    <col min="20" max="20" width="16.7109375" style="13" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.140625" style="15" customWidth="1"/>
+    <col min="18" max="18" width="8.81640625" style="13"/>
+    <col min="19" max="19" width="46.26953125" style="13" customWidth="1"/>
+    <col min="20" max="20" width="16.7265625" style="13" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.1796875" style="15" customWidth="1"/>
     <col min="22" max="22" width="11" style="15" customWidth="1"/>
-    <col min="23" max="23" width="11.140625" style="15" customWidth="1"/>
-    <col min="24" max="16384" width="8.85546875" style="4"/>
+    <col min="23" max="23" width="11.1796875" style="15" customWidth="1"/>
+    <col min="24" max="16384" width="8.81640625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:23" s="3" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C1" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="12" t="s">
         <v>18</v>
-      </c>
-      <c r="E1" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="12" t="s">
-        <v>19</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>10</v>
@@ -663,7 +600,7 @@
         <v>14</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>12</v>
@@ -672,10 +609,10 @@
         <v>13</v>
       </c>
       <c r="O1" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="P1" s="17" t="s">
         <v>22</v>
-      </c>
-      <c r="P1" s="17" t="s">
-        <v>23</v>
       </c>
       <c r="Q1" s="16" t="s">
         <v>1</v>
@@ -699,139 +636,27 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A2" s="10">
-        <v>46027</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="F2" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="I2" s="15">
-        <v>6482192</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="L2" s="4">
-        <v>1</v>
-      </c>
-      <c r="M2" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="N2" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="O2" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="P2" s="10">
-        <v>46027</v>
-      </c>
-      <c r="Q2" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="R2" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="S2" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="T2" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="U2" s="20">
-        <v>6482192</v>
-      </c>
-      <c r="V2" s="20">
-        <v>10</v>
-      </c>
-      <c r="W2" s="20">
-        <f>U2*10%</f>
-        <v>648219.20000000007</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A3" s="10">
-        <v>46027</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="F3" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="H3" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="I3" s="15">
-        <v>2997862</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="L3" s="4">
-        <v>1</v>
-      </c>
-      <c r="M3" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="N3" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="O3" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="P3" s="10">
-        <v>46027</v>
-      </c>
-      <c r="Q3" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="R3" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="S3" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="T3" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="U3" s="20">
-        <v>2997862</v>
-      </c>
-      <c r="V3" s="20">
-        <v>10</v>
-      </c>
-      <c r="W3" s="20">
-        <f>U3*10%</f>
-        <v>299786.2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A2" s="10"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="M2" s="5"/>
+      <c r="O2" s="18"/>
+      <c r="U2" s="20"/>
+      <c r="V2" s="20"/>
+      <c r="W2" s="20"/>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A3" s="10"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="M3" s="5"/>
+      <c r="O3" s="18"/>
+      <c r="U3" s="20"/>
+      <c r="V3" s="20"/>
+      <c r="W3" s="20"/>
+    </row>
+    <row r="4" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="10"/>
       <c r="G4" s="8"/>
       <c r="H4" s="8"/>
@@ -841,7 +666,7 @@
       <c r="V4" s="20"/>
       <c r="W4" s="20"/>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="10"/>
       <c r="G5" s="8"/>
       <c r="H5" s="8"/>
@@ -851,7 +676,7 @@
       <c r="V5" s="20"/>
       <c r="W5" s="20"/>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="10"/>
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
@@ -861,7 +686,7 @@
       <c r="V6" s="20"/>
       <c r="W6" s="20"/>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="10"/>
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
@@ -871,7 +696,7 @@
       <c r="V7" s="20"/>
       <c r="W7" s="20"/>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8" s="10"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
@@ -881,7 +706,7 @@
       <c r="V8" s="20"/>
       <c r="W8" s="20"/>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A9" s="10"/>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
@@ -891,7 +716,7 @@
       <c r="V9" s="20"/>
       <c r="W9" s="20"/>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A10" s="10"/>
       <c r="G10" s="8"/>
       <c r="H10" s="8"/>
@@ -901,7 +726,7 @@
       <c r="V10" s="20"/>
       <c r="W10" s="20"/>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A11" s="10"/>
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
@@ -911,7 +736,7 @@
       <c r="V11" s="20"/>
       <c r="W11" s="20"/>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A12" s="10"/>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
@@ -921,7 +746,7 @@
       <c r="V12" s="20"/>
       <c r="W12" s="20"/>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A13" s="10"/>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
@@ -931,7 +756,7 @@
       <c r="V13" s="20"/>
       <c r="W13" s="20"/>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A14" s="10"/>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
@@ -941,7 +766,7 @@
       <c r="V14" s="20"/>
       <c r="W14" s="20"/>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A15" s="10"/>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
@@ -951,7 +776,7 @@
       <c r="V15" s="20"/>
       <c r="W15" s="20"/>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A16" s="10"/>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
@@ -961,7 +786,7 @@
       <c r="V16" s="20"/>
       <c r="W16" s="20"/>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A17" s="10"/>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
@@ -971,7 +796,7 @@
       <c r="V17" s="20"/>
       <c r="W17" s="20"/>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A18" s="10"/>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
@@ -981,7 +806,7 @@
       <c r="V18" s="20"/>
       <c r="W18" s="20"/>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A19" s="10"/>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
@@ -991,7 +816,7 @@
       <c r="V19" s="20"/>
       <c r="W19" s="20"/>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A20" s="10"/>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
@@ -1001,7 +826,7 @@
       <c r="V20" s="20"/>
       <c r="W20" s="20"/>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A21" s="10"/>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
@@ -1011,7 +836,7 @@
       <c r="V21" s="20"/>
       <c r="W21" s="20"/>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A22" s="10"/>
       <c r="G22" s="8"/>
       <c r="H22" s="8"/>
@@ -1021,7 +846,7 @@
       <c r="V22" s="20"/>
       <c r="W22" s="20"/>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A23" s="10"/>
       <c r="G23" s="8"/>
       <c r="H23" s="8"/>
@@ -1031,7 +856,7 @@
       <c r="V23" s="20"/>
       <c r="W23" s="20"/>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A24" s="10"/>
       <c r="G24" s="8"/>
       <c r="H24" s="8"/>
@@ -1041,7 +866,7 @@
       <c r="V24" s="20"/>
       <c r="W24" s="20"/>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A25" s="10"/>
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
@@ -1051,7 +876,7 @@
       <c r="V25" s="20"/>
       <c r="W25" s="20"/>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A26" s="10"/>
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
@@ -1061,7 +886,7 @@
       <c r="V26" s="20"/>
       <c r="W26" s="20"/>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A27" s="10"/>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
@@ -1071,7 +896,7 @@
       <c r="V27" s="20"/>
       <c r="W27" s="20"/>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A28" s="10"/>
       <c r="G28" s="8"/>
       <c r="H28" s="8"/>
@@ -1081,7 +906,7 @@
       <c r="V28" s="20"/>
       <c r="W28" s="20"/>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A29" s="10"/>
       <c r="G29" s="8"/>
       <c r="H29" s="8"/>
@@ -1091,7 +916,7 @@
       <c r="V29" s="20"/>
       <c r="W29" s="20"/>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A30" s="10"/>
       <c r="G30" s="8"/>
       <c r="H30" s="8"/>
@@ -1101,7 +926,7 @@
       <c r="V30" s="20"/>
       <c r="W30" s="20"/>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A31" s="10"/>
       <c r="G31" s="8"/>
       <c r="H31" s="8"/>
@@ -1111,7 +936,7 @@
       <c r="V31" s="20"/>
       <c r="W31" s="20"/>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A32" s="10"/>
       <c r="G32" s="8"/>
       <c r="H32" s="8"/>
@@ -1121,7 +946,7 @@
       <c r="V32" s="20"/>
       <c r="W32" s="20"/>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A33" s="10"/>
       <c r="G33" s="8"/>
       <c r="H33" s="8"/>
@@ -1131,7 +956,7 @@
       <c r="V33" s="20"/>
       <c r="W33" s="20"/>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A34" s="10"/>
       <c r="G34" s="8"/>
       <c r="H34" s="8"/>
@@ -1141,7 +966,7 @@
       <c r="V34" s="20"/>
       <c r="W34" s="20"/>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A35" s="10"/>
       <c r="G35" s="8"/>
       <c r="H35" s="8"/>
@@ -1151,7 +976,7 @@
       <c r="V35" s="20"/>
       <c r="W35" s="20"/>
     </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A36" s="10"/>
       <c r="G36" s="8"/>
       <c r="H36" s="8"/>
@@ -1161,7 +986,7 @@
       <c r="V36" s="20"/>
       <c r="W36" s="20"/>
     </row>
-    <row r="37" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A37" s="10"/>
       <c r="G37" s="8"/>
       <c r="H37" s="8"/>
@@ -1171,7 +996,7 @@
       <c r="V37" s="20"/>
       <c r="W37" s="20"/>
     </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A38" s="10"/>
       <c r="G38" s="8"/>
       <c r="H38" s="8"/>
@@ -1181,7 +1006,7 @@
       <c r="V38" s="20"/>
       <c r="W38" s="20"/>
     </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A39" s="10"/>
       <c r="G39" s="8"/>
       <c r="H39" s="8"/>
@@ -1191,7 +1016,7 @@
       <c r="V39" s="20"/>
       <c r="W39" s="20"/>
     </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A40" s="10"/>
       <c r="G40" s="8"/>
       <c r="H40" s="8"/>
@@ -1201,7 +1026,7 @@
       <c r="V40" s="20"/>
       <c r="W40" s="20"/>
     </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A41" s="10"/>
       <c r="G41" s="8"/>
       <c r="H41" s="8"/>
@@ -1211,7 +1036,7 @@
       <c r="V41" s="20"/>
       <c r="W41" s="20"/>
     </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A42" s="10"/>
       <c r="G42" s="8"/>
       <c r="H42" s="8"/>
@@ -1221,7 +1046,7 @@
       <c r="V42" s="20"/>
       <c r="W42" s="20"/>
     </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A43" s="10"/>
       <c r="G43" s="8"/>
       <c r="H43" s="8"/>
@@ -1231,7 +1056,7 @@
       <c r="V43" s="20"/>
       <c r="W43" s="20"/>
     </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A44" s="10"/>
       <c r="G44" s="8"/>
       <c r="H44" s="8"/>
@@ -1241,7 +1066,7 @@
       <c r="V44" s="20"/>
       <c r="W44" s="20"/>
     </row>
-    <row r="45" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:23" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A45" s="10"/>
       <c r="G45" s="8"/>
       <c r="H45" s="8"/>
@@ -1251,7 +1076,7 @@
       <c r="V45" s="20"/>
       <c r="W45" s="20"/>
     </row>
-    <row r="46" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A46" s="10"/>
       <c r="G46" s="8"/>
       <c r="H46" s="8"/>
@@ -1261,7 +1086,7 @@
       <c r="V46" s="20"/>
       <c r="W46" s="20"/>
     </row>
-    <row r="47" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A47" s="10"/>
       <c r="G47" s="8"/>
       <c r="H47" s="8"/>
@@ -1271,7 +1096,7 @@
       <c r="V47" s="20"/>
       <c r="W47" s="20"/>
     </row>
-    <row r="48" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A48" s="10"/>
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
@@ -1281,7 +1106,7 @@
       <c r="V48" s="20"/>
       <c r="W48" s="20"/>
     </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A49" s="10"/>
       <c r="G49" s="8"/>
       <c r="H49" s="8"/>
@@ -1291,7 +1116,7 @@
       <c r="V49" s="20"/>
       <c r="W49" s="20"/>
     </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A50" s="10"/>
       <c r="G50" s="8"/>
       <c r="H50" s="8"/>
@@ -1301,7 +1126,7 @@
       <c r="V50" s="20"/>
       <c r="W50" s="20"/>
     </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A51" s="10"/>
       <c r="G51" s="8"/>
       <c r="H51" s="8"/>
@@ -1311,7 +1136,7 @@
       <c r="V51" s="20"/>
       <c r="W51" s="20"/>
     </row>
-    <row r="52" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A52" s="10"/>
       <c r="G52" s="8"/>
       <c r="H52" s="8"/>
@@ -1321,7 +1146,7 @@
       <c r="V52" s="20"/>
       <c r="W52" s="20"/>
     </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A53" s="10"/>
       <c r="G53" s="8"/>
       <c r="H53" s="8"/>
@@ -1331,7 +1156,7 @@
       <c r="V53" s="20"/>
       <c r="W53" s="20"/>
     </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A54" s="10"/>
       <c r="G54" s="8"/>
       <c r="H54" s="8"/>
@@ -1341,7 +1166,7 @@
       <c r="V54" s="20"/>
       <c r="W54" s="20"/>
     </row>
-    <row r="55" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A55" s="10"/>
       <c r="G55" s="8"/>
       <c r="H55" s="8"/>
@@ -1351,7 +1176,7 @@
       <c r="V55" s="20"/>
       <c r="W55" s="20"/>
     </row>
-    <row r="56" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A56" s="10"/>
       <c r="G56" s="8"/>
       <c r="H56" s="8"/>
@@ -1361,7 +1186,7 @@
       <c r="V56" s="20"/>
       <c r="W56" s="20"/>
     </row>
-    <row r="57" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A57" s="10"/>
       <c r="G57" s="8"/>
       <c r="H57" s="8"/>
@@ -1371,7 +1196,7 @@
       <c r="V57" s="20"/>
       <c r="W57" s="20"/>
     </row>
-    <row r="58" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A58" s="10"/>
       <c r="G58" s="8"/>
       <c r="H58" s="8"/>
@@ -1381,7 +1206,7 @@
       <c r="V58" s="20"/>
       <c r="W58" s="20"/>
     </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A59" s="10"/>
       <c r="G59" s="8"/>
       <c r="H59" s="8"/>
@@ -1391,7 +1216,7 @@
       <c r="V59" s="20"/>
       <c r="W59" s="20"/>
     </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A60" s="10"/>
       <c r="G60" s="8"/>
       <c r="H60" s="8"/>
@@ -1401,7 +1226,7 @@
       <c r="V60" s="20"/>
       <c r="W60" s="20"/>
     </row>
-    <row r="61" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A61" s="10"/>
       <c r="G61" s="8"/>
       <c r="H61" s="8"/>
@@ -1411,7 +1236,7 @@
       <c r="V61" s="20"/>
       <c r="W61" s="20"/>
     </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A62" s="10"/>
       <c r="G62" s="8"/>
       <c r="H62" s="8"/>
@@ -1421,7 +1246,7 @@
       <c r="V62" s="20"/>
       <c r="W62" s="20"/>
     </row>
-    <row r="63" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A63" s="10"/>
       <c r="G63" s="8"/>
       <c r="H63" s="8"/>
@@ -1431,7 +1256,7 @@
       <c r="V63" s="20"/>
       <c r="W63" s="20"/>
     </row>
-    <row r="64" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A64" s="10"/>
       <c r="G64" s="8"/>
       <c r="H64" s="8"/>
@@ -1441,7 +1266,7 @@
       <c r="V64" s="20"/>
       <c r="W64" s="20"/>
     </row>
-    <row r="65" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A65" s="10"/>
       <c r="G65" s="8"/>
       <c r="H65" s="8"/>
@@ -1451,7 +1276,7 @@
       <c r="V65" s="20"/>
       <c r="W65" s="20"/>
     </row>
-    <row r="66" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A66" s="10"/>
       <c r="G66" s="8"/>
       <c r="H66" s="8"/>
@@ -1461,7 +1286,7 @@
       <c r="V66" s="20"/>
       <c r="W66" s="20"/>
     </row>
-    <row r="67" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A67" s="10"/>
       <c r="G67" s="8"/>
       <c r="H67" s="8"/>
@@ -1471,7 +1296,7 @@
       <c r="V67" s="20"/>
       <c r="W67" s="20"/>
     </row>
-    <row r="68" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A68" s="10"/>
       <c r="G68" s="8"/>
       <c r="H68" s="8"/>
@@ -1481,7 +1306,7 @@
       <c r="V68" s="20"/>
       <c r="W68" s="20"/>
     </row>
-    <row r="69" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A69" s="10"/>
       <c r="G69" s="8"/>
       <c r="H69" s="8"/>
@@ -1491,7 +1316,7 @@
       <c r="V69" s="20"/>
       <c r="W69" s="20"/>
     </row>
-    <row r="70" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A70" s="10"/>
       <c r="G70" s="8"/>
       <c r="H70" s="8"/>
@@ -1501,7 +1326,7 @@
       <c r="V70" s="20"/>
       <c r="W70" s="20"/>
     </row>
-    <row r="71" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A71" s="10"/>
       <c r="G71" s="8"/>
       <c r="H71" s="8"/>
@@ -1511,7 +1336,7 @@
       <c r="V71" s="20"/>
       <c r="W71" s="20"/>
     </row>
-    <row r="72" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A72" s="10"/>
       <c r="G72" s="8"/>
       <c r="H72" s="8"/>
@@ -1521,7 +1346,7 @@
       <c r="V72" s="20"/>
       <c r="W72" s="20"/>
     </row>
-    <row r="73" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A73" s="10"/>
       <c r="G73" s="8"/>
       <c r="H73" s="8"/>
@@ -1531,7 +1356,7 @@
       <c r="V73" s="20"/>
       <c r="W73" s="20"/>
     </row>
-    <row r="74" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A74" s="10"/>
       <c r="G74" s="8"/>
       <c r="H74" s="8"/>
@@ -1541,7 +1366,7 @@
       <c r="V74" s="20"/>
       <c r="W74" s="20"/>
     </row>
-    <row r="75" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A75" s="10"/>
       <c r="G75" s="8"/>
       <c r="H75" s="8"/>
@@ -1551,7 +1376,7 @@
       <c r="V75" s="20"/>
       <c r="W75" s="20"/>
     </row>
-    <row r="76" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A76" s="10"/>
       <c r="G76" s="8"/>
       <c r="H76" s="8"/>
@@ -1561,7 +1386,7 @@
       <c r="V76" s="20"/>
       <c r="W76" s="20"/>
     </row>
-    <row r="77" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A77" s="10"/>
       <c r="G77" s="8"/>
       <c r="H77" s="8"/>
@@ -1571,7 +1396,7 @@
       <c r="V77" s="20"/>
       <c r="W77" s="20"/>
     </row>
-    <row r="78" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A78" s="10"/>
       <c r="G78" s="8"/>
       <c r="H78" s="8"/>
@@ -1581,7 +1406,7 @@
       <c r="V78" s="20"/>
       <c r="W78" s="20"/>
     </row>
-    <row r="79" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A79" s="10"/>
       <c r="G79" s="8"/>
       <c r="H79" s="8"/>
@@ -1591,7 +1416,7 @@
       <c r="V79" s="20"/>
       <c r="W79" s="20"/>
     </row>
-    <row r="80" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A80" s="10"/>
       <c r="G80" s="8"/>
       <c r="H80" s="8"/>
@@ -1601,7 +1426,7 @@
       <c r="V80" s="20"/>
       <c r="W80" s="20"/>
     </row>
-    <row r="81" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A81" s="10"/>
       <c r="G81" s="8"/>
       <c r="H81" s="8"/>
@@ -1611,7 +1436,7 @@
       <c r="V81" s="20"/>
       <c r="W81" s="20"/>
     </row>
-    <row r="82" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A82" s="10"/>
       <c r="G82" s="8"/>
       <c r="H82" s="8"/>
@@ -1621,7 +1446,7 @@
       <c r="V82" s="20"/>
       <c r="W82" s="20"/>
     </row>
-    <row r="83" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A83" s="10"/>
       <c r="G83" s="8"/>
       <c r="H83" s="8"/>
@@ -1631,7 +1456,7 @@
       <c r="V83" s="20"/>
       <c r="W83" s="20"/>
     </row>
-    <row r="84" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A84" s="10"/>
       <c r="G84" s="8"/>
       <c r="H84" s="8"/>
@@ -1641,7 +1466,7 @@
       <c r="V84" s="20"/>
       <c r="W84" s="20"/>
     </row>
-    <row r="85" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A85" s="10"/>
       <c r="G85" s="8"/>
       <c r="H85" s="8"/>
@@ -1651,7 +1476,7 @@
       <c r="V85" s="20"/>
       <c r="W85" s="20"/>
     </row>
-    <row r="86" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A86" s="10"/>
       <c r="G86" s="8"/>
       <c r="H86" s="8"/>
@@ -1661,7 +1486,7 @@
       <c r="V86" s="20"/>
       <c r="W86" s="20"/>
     </row>
-    <row r="87" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A87" s="10"/>
       <c r="G87" s="8"/>
       <c r="H87" s="8"/>
@@ -1671,7 +1496,7 @@
       <c r="V87" s="20"/>
       <c r="W87" s="20"/>
     </row>
-    <row r="88" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A88" s="10"/>
       <c r="G88" s="8"/>
       <c r="H88" s="8"/>
@@ -1681,7 +1506,7 @@
       <c r="V88" s="20"/>
       <c r="W88" s="20"/>
     </row>
-    <row r="89" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A89" s="10"/>
       <c r="G89" s="8"/>
       <c r="H89" s="8"/>
@@ -1691,7 +1516,7 @@
       <c r="V89" s="20"/>
       <c r="W89" s="20"/>
     </row>
-    <row r="90" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A90" s="10"/>
       <c r="G90" s="8"/>
       <c r="H90" s="8"/>
@@ -1701,7 +1526,7 @@
       <c r="V90" s="20"/>
       <c r="W90" s="20"/>
     </row>
-    <row r="91" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A91" s="10"/>
       <c r="G91" s="8"/>
       <c r="H91" s="8"/>
@@ -1711,7 +1536,7 @@
       <c r="V91" s="20"/>
       <c r="W91" s="20"/>
     </row>
-    <row r="92" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A92" s="10"/>
       <c r="G92" s="8"/>
       <c r="H92" s="8"/>
@@ -1721,7 +1546,7 @@
       <c r="V92" s="20"/>
       <c r="W92" s="20"/>
     </row>
-    <row r="93" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A93" s="10"/>
       <c r="G93" s="8"/>
       <c r="H93" s="8"/>
@@ -1731,7 +1556,7 @@
       <c r="V93" s="20"/>
       <c r="W93" s="20"/>
     </row>
-    <row r="94" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A94" s="10"/>
       <c r="G94" s="8"/>
       <c r="H94" s="8"/>
@@ -1741,7 +1566,7 @@
       <c r="V94" s="20"/>
       <c r="W94" s="20"/>
     </row>
-    <row r="95" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A95" s="10"/>
       <c r="G95" s="8"/>
       <c r="H95" s="8"/>
@@ -1751,7 +1576,7 @@
       <c r="V95" s="20"/>
       <c r="W95" s="20"/>
     </row>
-    <row r="96" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A96" s="10"/>
       <c r="G96" s="8"/>
       <c r="H96" s="8"/>
@@ -1761,7 +1586,7 @@
       <c r="V96" s="20"/>
       <c r="W96" s="20"/>
     </row>
-    <row r="97" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A97" s="10"/>
       <c r="G97" s="8"/>
       <c r="H97" s="8"/>
@@ -1771,7 +1596,7 @@
       <c r="V97" s="20"/>
       <c r="W97" s="20"/>
     </row>
-    <row r="98" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A98" s="10"/>
       <c r="G98" s="8"/>
       <c r="H98" s="8"/>
@@ -1781,7 +1606,7 @@
       <c r="V98" s="20"/>
       <c r="W98" s="20"/>
     </row>
-    <row r="99" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A99" s="10"/>
       <c r="G99" s="8"/>
       <c r="H99" s="8"/>
@@ -1791,7 +1616,7 @@
       <c r="V99" s="20"/>
       <c r="W99" s="20"/>
     </row>
-    <row r="100" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A100" s="10"/>
       <c r="G100" s="8"/>
       <c r="H100" s="8"/>
@@ -1801,7 +1626,7 @@
       <c r="V100" s="20"/>
       <c r="W100" s="20"/>
     </row>
-    <row r="101" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A101" s="10"/>
       <c r="G101" s="8"/>
       <c r="H101" s="8"/>
@@ -1811,7 +1636,7 @@
       <c r="V101" s="20"/>
       <c r="W101" s="20"/>
     </row>
-    <row r="102" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A102" s="10"/>
       <c r="G102" s="8"/>
       <c r="H102" s="8"/>
@@ -1821,7 +1646,7 @@
       <c r="V102" s="20"/>
       <c r="W102" s="20"/>
     </row>
-    <row r="103" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A103" s="10"/>
       <c r="G103" s="8"/>
       <c r="H103" s="8"/>
@@ -1831,7 +1656,7 @@
       <c r="V103" s="20"/>
       <c r="W103" s="20"/>
     </row>
-    <row r="104" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A104" s="10"/>
       <c r="G104" s="8"/>
       <c r="H104" s="8"/>
@@ -1841,7 +1666,7 @@
       <c r="V104" s="20"/>
       <c r="W104" s="20"/>
     </row>
-    <row r="105" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A105" s="10"/>
       <c r="G105" s="8"/>
       <c r="H105" s="8"/>
@@ -1851,7 +1676,7 @@
       <c r="V105" s="20"/>
       <c r="W105" s="20"/>
     </row>
-    <row r="106" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A106" s="10"/>
       <c r="G106" s="8"/>
       <c r="H106" s="8"/>
@@ -1862,7 +1687,7 @@
       <c r="W106" s="20"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:W3">
+  <sortState ref="A2:W3">
     <sortCondition ref="A2:A3"/>
   </sortState>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>